<commit_message>
added input list 0 or 1
</commit_message>
<xml_diff>
--- a/7SegPortasLogicas.xlsx
+++ b/7SegPortasLogicas.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29115"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Imperio\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{32EA32F8-C20B-43AE-B7CA-6E31717936D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE3D024-CA80-4DB5-BC01-21DD5115FE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16395" yWindow="0" windowWidth="11745" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="7 Segmentos Binário" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>AND</t>
   </si>
@@ -58,6 +57,9 @@
   </si>
   <si>
     <t>z</t>
+  </si>
+  <si>
+    <t>input</t>
   </si>
 </sst>
 </file>
@@ -109,12 +111,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -446,7 +447,7 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
+      <c r="A2" s="2"/>
       <c r="B2" t="str">
         <f>IF(A1="", "", IF(ISNUMBER(FIND(A1, "045689")), 1, ""))</f>
         <v/>
@@ -533,10 +534,9 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="1"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="G6">
         <v>0</v>
       </c>
@@ -679,7 +679,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J13" s="3"/>
+      <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -712,7 +712,7 @@
         <f>DEC2BIN(C16)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <f>SUM(C7:C15)</f>
         <v>0</v>
       </c>
@@ -783,7 +783,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D19" s="3"/>
+      <c r="D19" s="2"/>
       <c r="E19">
         <f>IF(D18="", "", IF(ISNUMBER(FIND(D18, "045689")), 1, ""))</f>
         <v>1</v>
@@ -792,7 +792,7 @@
         <f>IF(D18="", "", IF(ISNUMBER(FIND(D18, "01234789")), 1, ""))</f>
         <v>1</v>
       </c>
-      <c r="H19" s="3"/>
+      <c r="H19" s="2"/>
       <c r="I19" t="str">
         <f>IF(H18="", "", IF(ISNUMBER(FIND(H18, "045689")), 1, ""))</f>
         <v/>
@@ -801,7 +801,7 @@
         <f>IF(H18="", "", IF(ISNUMBER(FIND(H18, "01234789")), 1, ""))</f>
         <v/>
       </c>
-      <c r="L19" s="3"/>
+      <c r="L19" s="2"/>
       <c r="M19" t="str">
         <f>IF(L18="", "", IF(ISNUMBER(FIND(L18, "045689")), 1, ""))</f>
         <v/>
@@ -920,7 +920,7 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
+      <c r="A24" s="2"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -948,7 +948,7 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
+      <c r="A26" s="2"/>
       <c r="B26" t="str">
         <f>IF(A25="", "", IF(ISNUMBER(FIND(A25, "045689abcdefghklmnopqrsuvwxy")), 1, ""))</f>
         <v/>
@@ -1039,8 +1039,56 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color theme="0"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:D29">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color theme="0"/>
+        <color theme="1"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D6:F8 B1:D5">
     <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color theme="0"/>
+        <color theme="1"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:E29">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color theme="0"/>
+        <color theme="1"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:F25">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1056,6 +1104,34 @@
         <cfvo type="num" val="1"/>
         <color theme="0"/>
         <color theme="1"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F26:F29">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <color theme="0"/>
+        <color theme="1"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color theme="0"/>
+        <color rgb="FF92D050"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -1079,82 +1155,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0"/>
-        <color rgb="FF92D050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25:D29">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0"/>
-        <color theme="1"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E25:F25">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0"/>
-        <color theme="1"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E26:E29">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color theme="0"/>
-        <color theme="1"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F26:F29">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <color theme="0"/>
-        <color theme="1"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B15 G6:G7 G2:G3 G10:G11 J3 J6:J7 M6:M7 M2:M3" xr:uid="{50B616C5-B1D7-4F3E-9504-0565E3BE49A2}">
+      <formula1>"0,1"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>